<commit_message>
Expand product details and hide empty tabs
</commit_message>
<xml_diff>
--- a/outputs/product-import/HLC_产品资料导入表.xlsx
+++ b/outputs/product-import/HLC_产品资料导入表.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R3f9d0320f7604a66"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品基础信息" sheetId="2" r:id="Rf0d1d150c6d4491a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品内容与SEO" sheetId="3" r:id="R047403fc153642b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品图片" sheetId="4" r:id="Rff619b64c21e4f4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="相关产品" sheetId="5" r:id="R9935e4ca9a9c4ba0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="Rba82ff3529084a89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品基础信息" sheetId="2" r:id="Rf88c3e2912484a8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品内容与SEO" sheetId="3" r:id="R3c89a1a0fc7c4b0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品图片" sheetId="4" r:id="Rca78a4b2de0d4cbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="相关产品" sheetId="5" r:id="R4a97072de49643bb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -270,8 +270,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ProductBasicsTable" displayName="ProductBasicsTable" ref="A4:V104" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="22">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ProductBasicsTable" displayName="ProductBasicsTable" ref="A4:X104" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="24">
     <x:tableColumn id="1" name="发布"/>
     <x:tableColumn id="2" name="产品URL标识"/>
     <x:tableColumn id="3" name="款号（Style#）"/>
@@ -288,12 +288,14 @@
     <x:tableColumn id="14" name="纱支"/>
     <x:tableColumn id="15" name="后整理"/>
     <x:tableColumn id="16" name="起订量 / 单色起订量"/>
-    <x:tableColumn id="17" name="适用产品"/>
-    <x:tableColumn id="18" name="HS编码（选填）"/>
-    <x:tableColumn id="19" name="原产国"/>
-    <x:tableColumn id="20" name="完整URL（自动）"/>
-    <x:tableColumn id="21" name="资料检查（自动）"/>
-    <x:tableColumn id="22" name="备注（不发布）"/>
+    <x:tableColumn id="17" name="样品交期（英文）"/>
+    <x:tableColumn id="18" name="大货交期（英文）"/>
+    <x:tableColumn id="19" name="适用产品"/>
+    <x:tableColumn id="20" name="HS编码（选填）"/>
+    <x:tableColumn id="21" name="原产国"/>
+    <x:tableColumn id="22" name="完整URL（自动）"/>
+    <x:tableColumn id="23" name="资料检查（自动）"/>
+    <x:tableColumn id="24" name="备注（不发布）"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -829,12 +831,14 @@
     <x:col min="14" max="14" width="18" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="24" hidden="0" customWidth="1"/>
     <x:col min="16" max="16" width="24" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="34" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="18" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="14" hidden="0" customWidth="1"/>
-    <x:col min="20" max="20" width="45" hidden="0" customWidth="1"/>
-    <x:col min="21" max="21" width="18" hidden="0" customWidth="1"/>
-    <x:col min="22" max="22" width="34" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="22" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="24" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="34" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="18" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="14" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="45" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="18" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="34" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -862,6 +866,8 @@
       <x:c r="T1" s="4"/>
       <x:c r="U1" s="4"/>
       <x:c r="V1" s="4"/>
+      <x:c r="W1" s="4"/>
+      <x:c r="X1" s="4"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="8" t="str">
@@ -888,6 +894,8 @@
       <x:c r="T2" s="8"/>
       <x:c r="U2" s="8"/>
       <x:c r="V2" s="8"/>
+      <x:c r="W2" s="8"/>
+      <x:c r="X2" s="8"/>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
       <x:c r="A4" s="30" t="str">
@@ -939,21 +947,27 @@
         <x:v>起订量 / 单色起订量</x:v>
       </x:c>
       <x:c r="Q4" s="30" t="str">
+        <x:v>样品交期（英文）</x:v>
+      </x:c>
+      <x:c r="R4" s="30" t="str">
+        <x:v>大货交期（英文）</x:v>
+      </x:c>
+      <x:c r="S4" s="30" t="str">
         <x:v>适用产品</x:v>
       </x:c>
-      <x:c r="R4" s="30" t="str">
+      <x:c r="T4" s="30" t="str">
         <x:v>HS编码（选填）</x:v>
       </x:c>
-      <x:c r="S4" s="30" t="str">
+      <x:c r="U4" s="30" t="str">
         <x:v>原产国</x:v>
       </x:c>
-      <x:c r="T4" s="30" t="str">
+      <x:c r="V4" s="30" t="str">
         <x:v>完整URL（自动）</x:v>
       </x:c>
-      <x:c r="U4" s="30" t="str">
+      <x:c r="W4" s="30" t="str">
         <x:v>资料检查（自动）</x:v>
       </x:c>
-      <x:c r="V4" s="30" t="str">
+      <x:c r="X4" s="30" t="str">
         <x:v>备注（不发布）</x:v>
       </x:c>
     </x:row>
@@ -1007,23 +1021,29 @@
         <x:v>500 kg / 100 kg per colour</x:v>
       </x:c>
       <x:c r="Q5" s="36" t="str">
+        <x:v>5–7 working days</x:v>
+      </x:c>
+      <x:c r="R5" s="36" t="str">
+        <x:v>25–35 days after approval</x:v>
+      </x:c>
+      <x:c r="S5" s="36" t="str">
         <x:v>Babywear, sleepwear and loungewear</x:v>
       </x:c>
-      <x:c r="R5" s="36" t="str">
+      <x:c r="T5" s="36" t="str">
         <x:v>6006.32</x:v>
       </x:c>
-      <x:c r="S5" s="36" t="str">
+      <x:c r="U5" s="36" t="str">
         <x:v>China</x:v>
       </x:c>
-      <x:c r="T5" s="38" t="str">
+      <x:c r="V5" s="38" t="str">
         <x:f>IF(B5="","","https://hlctex.com/textile/products/"&amp;B5&amp;"/")</x:f>
         <x:v>https://hlctex.com/textile/products/example-bamboo-knit/</x:v>
       </x:c>
-      <x:c r="U5" s="38" t="str">
+      <x:c r="W5" s="38" t="str">
         <x:f>IF(B5="","",IF(A5&lt;&gt;"YES","未发布",IF(OR(C5="",D5="",J5=""),"缺少必填项","可生成")))</x:f>
         <x:v>未发布</x:v>
       </x:c>
-      <x:c r="V5" s="36" t="str">
+      <x:c r="X5" s="36" t="str">
         <x:v>示例行，请复制后填写真实产品</x:v>
       </x:c>
     </x:row>
@@ -1047,13 +1067,15 @@
       <x:c r="Q6" s="36"/>
       <x:c r="R6" s="36"/>
       <x:c r="S6" s="36"/>
-      <x:c r="T6" s="38" t="str">
+      <x:c r="T6" s="36"/>
+      <x:c r="U6" s="36"/>
+      <x:c r="V6" s="38" t="str">
         <x:f>IF(B6="","","https://hlctex.com/textile/products/"&amp;B6&amp;"/")</x:f>
       </x:c>
-      <x:c r="U6" s="38" t="str">
+      <x:c r="W6" s="38" t="str">
         <x:f>IF(B6="","",IF(A6&lt;&gt;"YES","未发布",IF(OR(C6="",D6="",J6=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V6" s="36"/>
+      <x:c r="X6" s="36"/>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
       <x:c r="A7" s="36"/>
@@ -1075,13 +1097,15 @@
       <x:c r="Q7" s="36"/>
       <x:c r="R7" s="36"/>
       <x:c r="S7" s="36"/>
-      <x:c r="T7" s="38" t="str">
+      <x:c r="T7" s="36"/>
+      <x:c r="U7" s="36"/>
+      <x:c r="V7" s="38" t="str">
         <x:f>IF(B7="","","https://hlctex.com/textile/products/"&amp;B7&amp;"/")</x:f>
       </x:c>
-      <x:c r="U7" s="38" t="str">
+      <x:c r="W7" s="38" t="str">
         <x:f>IF(B7="","",IF(A7&lt;&gt;"YES","未发布",IF(OR(C7="",D7="",J7=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V7" s="36"/>
+      <x:c r="X7" s="36"/>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
       <x:c r="A8" s="36"/>
@@ -1103,13 +1127,15 @@
       <x:c r="Q8" s="36"/>
       <x:c r="R8" s="36"/>
       <x:c r="S8" s="36"/>
-      <x:c r="T8" s="38" t="str">
+      <x:c r="T8" s="36"/>
+      <x:c r="U8" s="36"/>
+      <x:c r="V8" s="38" t="str">
         <x:f>IF(B8="","","https://hlctex.com/textile/products/"&amp;B8&amp;"/")</x:f>
       </x:c>
-      <x:c r="U8" s="38" t="str">
+      <x:c r="W8" s="38" t="str">
         <x:f>IF(B8="","",IF(A8&lt;&gt;"YES","未发布",IF(OR(C8="",D8="",J8=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V8" s="36"/>
+      <x:c r="X8" s="36"/>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
       <x:c r="A9" s="36"/>
@@ -1131,13 +1157,15 @@
       <x:c r="Q9" s="36"/>
       <x:c r="R9" s="36"/>
       <x:c r="S9" s="36"/>
-      <x:c r="T9" s="38" t="str">
+      <x:c r="T9" s="36"/>
+      <x:c r="U9" s="36"/>
+      <x:c r="V9" s="38" t="str">
         <x:f>IF(B9="","","https://hlctex.com/textile/products/"&amp;B9&amp;"/")</x:f>
       </x:c>
-      <x:c r="U9" s="38" t="str">
+      <x:c r="W9" s="38" t="str">
         <x:f>IF(B9="","",IF(A9&lt;&gt;"YES","未发布",IF(OR(C9="",D9="",J9=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V9" s="36"/>
+      <x:c r="X9" s="36"/>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
       <x:c r="A10" s="36"/>
@@ -1159,13 +1187,15 @@
       <x:c r="Q10" s="36"/>
       <x:c r="R10" s="36"/>
       <x:c r="S10" s="36"/>
-      <x:c r="T10" s="38" t="str">
+      <x:c r="T10" s="36"/>
+      <x:c r="U10" s="36"/>
+      <x:c r="V10" s="38" t="str">
         <x:f>IF(B10="","","https://hlctex.com/textile/products/"&amp;B10&amp;"/")</x:f>
       </x:c>
-      <x:c r="U10" s="38" t="str">
+      <x:c r="W10" s="38" t="str">
         <x:f>IF(B10="","",IF(A10&lt;&gt;"YES","未发布",IF(OR(C10="",D10="",J10=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V10" s="36"/>
+      <x:c r="X10" s="36"/>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
       <x:c r="A11" s="36"/>
@@ -1187,13 +1217,15 @@
       <x:c r="Q11" s="36"/>
       <x:c r="R11" s="36"/>
       <x:c r="S11" s="36"/>
-      <x:c r="T11" s="38" t="str">
+      <x:c r="T11" s="36"/>
+      <x:c r="U11" s="36"/>
+      <x:c r="V11" s="38" t="str">
         <x:f>IF(B11="","","https://hlctex.com/textile/products/"&amp;B11&amp;"/")</x:f>
       </x:c>
-      <x:c r="U11" s="38" t="str">
+      <x:c r="W11" s="38" t="str">
         <x:f>IF(B11="","",IF(A11&lt;&gt;"YES","未发布",IF(OR(C11="",D11="",J11=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V11" s="36"/>
+      <x:c r="X11" s="36"/>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="36"/>
@@ -1215,13 +1247,15 @@
       <x:c r="Q12" s="36"/>
       <x:c r="R12" s="36"/>
       <x:c r="S12" s="36"/>
-      <x:c r="T12" s="38" t="str">
+      <x:c r="T12" s="36"/>
+      <x:c r="U12" s="36"/>
+      <x:c r="V12" s="38" t="str">
         <x:f>IF(B12="","","https://hlctex.com/textile/products/"&amp;B12&amp;"/")</x:f>
       </x:c>
-      <x:c r="U12" s="38" t="str">
+      <x:c r="W12" s="38" t="str">
         <x:f>IF(B12="","",IF(A12&lt;&gt;"YES","未发布",IF(OR(C12="",D12="",J12=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V12" s="36"/>
+      <x:c r="X12" s="36"/>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
       <x:c r="A13" s="36"/>
@@ -1243,13 +1277,15 @@
       <x:c r="Q13" s="36"/>
       <x:c r="R13" s="36"/>
       <x:c r="S13" s="36"/>
-      <x:c r="T13" s="38" t="str">
+      <x:c r="T13" s="36"/>
+      <x:c r="U13" s="36"/>
+      <x:c r="V13" s="38" t="str">
         <x:f>IF(B13="","","https://hlctex.com/textile/products/"&amp;B13&amp;"/")</x:f>
       </x:c>
-      <x:c r="U13" s="38" t="str">
+      <x:c r="W13" s="38" t="str">
         <x:f>IF(B13="","",IF(A13&lt;&gt;"YES","未发布",IF(OR(C13="",D13="",J13=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V13" s="36"/>
+      <x:c r="X13" s="36"/>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
       <x:c r="A14" s="36"/>
@@ -1271,13 +1307,15 @@
       <x:c r="Q14" s="36"/>
       <x:c r="R14" s="36"/>
       <x:c r="S14" s="36"/>
-      <x:c r="T14" s="38" t="str">
+      <x:c r="T14" s="36"/>
+      <x:c r="U14" s="36"/>
+      <x:c r="V14" s="38" t="str">
         <x:f>IF(B14="","","https://hlctex.com/textile/products/"&amp;B14&amp;"/")</x:f>
       </x:c>
-      <x:c r="U14" s="38" t="str">
+      <x:c r="W14" s="38" t="str">
         <x:f>IF(B14="","",IF(A14&lt;&gt;"YES","未发布",IF(OR(C14="",D14="",J14=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V14" s="36"/>
+      <x:c r="X14" s="36"/>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
       <x:c r="A15" s="36"/>
@@ -1299,13 +1337,15 @@
       <x:c r="Q15" s="36"/>
       <x:c r="R15" s="36"/>
       <x:c r="S15" s="36"/>
-      <x:c r="T15" s="38" t="str">
+      <x:c r="T15" s="36"/>
+      <x:c r="U15" s="36"/>
+      <x:c r="V15" s="38" t="str">
         <x:f>IF(B15="","","https://hlctex.com/textile/products/"&amp;B15&amp;"/")</x:f>
       </x:c>
-      <x:c r="U15" s="38" t="str">
+      <x:c r="W15" s="38" t="str">
         <x:f>IF(B15="","",IF(A15&lt;&gt;"YES","未发布",IF(OR(C15="",D15="",J15=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V15" s="36"/>
+      <x:c r="X15" s="36"/>
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
       <x:c r="A16" s="36"/>
@@ -1327,13 +1367,15 @@
       <x:c r="Q16" s="36"/>
       <x:c r="R16" s="36"/>
       <x:c r="S16" s="36"/>
-      <x:c r="T16" s="38" t="str">
+      <x:c r="T16" s="36"/>
+      <x:c r="U16" s="36"/>
+      <x:c r="V16" s="38" t="str">
         <x:f>IF(B16="","","https://hlctex.com/textile/products/"&amp;B16&amp;"/")</x:f>
       </x:c>
-      <x:c r="U16" s="38" t="str">
+      <x:c r="W16" s="38" t="str">
         <x:f>IF(B16="","",IF(A16&lt;&gt;"YES","未发布",IF(OR(C16="",D16="",J16=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V16" s="36"/>
+      <x:c r="X16" s="36"/>
     </x:row>
     <x:row r="17" ht="42" customHeight="1">
       <x:c r="A17" s="36"/>
@@ -1355,13 +1397,15 @@
       <x:c r="Q17" s="36"/>
       <x:c r="R17" s="36"/>
       <x:c r="S17" s="36"/>
-      <x:c r="T17" s="38" t="str">
+      <x:c r="T17" s="36"/>
+      <x:c r="U17" s="36"/>
+      <x:c r="V17" s="38" t="str">
         <x:f>IF(B17="","","https://hlctex.com/textile/products/"&amp;B17&amp;"/")</x:f>
       </x:c>
-      <x:c r="U17" s="38" t="str">
+      <x:c r="W17" s="38" t="str">
         <x:f>IF(B17="","",IF(A17&lt;&gt;"YES","未发布",IF(OR(C17="",D17="",J17=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V17" s="36"/>
+      <x:c r="X17" s="36"/>
     </x:row>
     <x:row r="18" ht="42" customHeight="1">
       <x:c r="A18" s="36"/>
@@ -1383,13 +1427,15 @@
       <x:c r="Q18" s="36"/>
       <x:c r="R18" s="36"/>
       <x:c r="S18" s="36"/>
-      <x:c r="T18" s="38" t="str">
+      <x:c r="T18" s="36"/>
+      <x:c r="U18" s="36"/>
+      <x:c r="V18" s="38" t="str">
         <x:f>IF(B18="","","https://hlctex.com/textile/products/"&amp;B18&amp;"/")</x:f>
       </x:c>
-      <x:c r="U18" s="38" t="str">
+      <x:c r="W18" s="38" t="str">
         <x:f>IF(B18="","",IF(A18&lt;&gt;"YES","未发布",IF(OR(C18="",D18="",J18=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V18" s="36"/>
+      <x:c r="X18" s="36"/>
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
       <x:c r="A19" s="36"/>
@@ -1411,13 +1457,15 @@
       <x:c r="Q19" s="36"/>
       <x:c r="R19" s="36"/>
       <x:c r="S19" s="36"/>
-      <x:c r="T19" s="38" t="str">
+      <x:c r="T19" s="36"/>
+      <x:c r="U19" s="36"/>
+      <x:c r="V19" s="38" t="str">
         <x:f>IF(B19="","","https://hlctex.com/textile/products/"&amp;B19&amp;"/")</x:f>
       </x:c>
-      <x:c r="U19" s="38" t="str">
+      <x:c r="W19" s="38" t="str">
         <x:f>IF(B19="","",IF(A19&lt;&gt;"YES","未发布",IF(OR(C19="",D19="",J19=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V19" s="36"/>
+      <x:c r="X19" s="36"/>
     </x:row>
     <x:row r="20" ht="42" customHeight="1">
       <x:c r="A20" s="36"/>
@@ -1439,13 +1487,15 @@
       <x:c r="Q20" s="36"/>
       <x:c r="R20" s="36"/>
       <x:c r="S20" s="36"/>
-      <x:c r="T20" s="38" t="str">
+      <x:c r="T20" s="36"/>
+      <x:c r="U20" s="36"/>
+      <x:c r="V20" s="38" t="str">
         <x:f>IF(B20="","","https://hlctex.com/textile/products/"&amp;B20&amp;"/")</x:f>
       </x:c>
-      <x:c r="U20" s="38" t="str">
+      <x:c r="W20" s="38" t="str">
         <x:f>IF(B20="","",IF(A20&lt;&gt;"YES","未发布",IF(OR(C20="",D20="",J20=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V20" s="36"/>
+      <x:c r="X20" s="36"/>
     </x:row>
     <x:row r="21" ht="42" customHeight="1">
       <x:c r="A21" s="36"/>
@@ -1467,13 +1517,15 @@
       <x:c r="Q21" s="36"/>
       <x:c r="R21" s="36"/>
       <x:c r="S21" s="36"/>
-      <x:c r="T21" s="38" t="str">
+      <x:c r="T21" s="36"/>
+      <x:c r="U21" s="36"/>
+      <x:c r="V21" s="38" t="str">
         <x:f>IF(B21="","","https://hlctex.com/textile/products/"&amp;B21&amp;"/")</x:f>
       </x:c>
-      <x:c r="U21" s="38" t="str">
+      <x:c r="W21" s="38" t="str">
         <x:f>IF(B21="","",IF(A21&lt;&gt;"YES","未发布",IF(OR(C21="",D21="",J21=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V21" s="36"/>
+      <x:c r="X21" s="36"/>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
       <x:c r="A22" s="36"/>
@@ -1495,13 +1547,15 @@
       <x:c r="Q22" s="36"/>
       <x:c r="R22" s="36"/>
       <x:c r="S22" s="36"/>
-      <x:c r="T22" s="38" t="str">
+      <x:c r="T22" s="36"/>
+      <x:c r="U22" s="36"/>
+      <x:c r="V22" s="38" t="str">
         <x:f>IF(B22="","","https://hlctex.com/textile/products/"&amp;B22&amp;"/")</x:f>
       </x:c>
-      <x:c r="U22" s="38" t="str">
+      <x:c r="W22" s="38" t="str">
         <x:f>IF(B22="","",IF(A22&lt;&gt;"YES","未发布",IF(OR(C22="",D22="",J22=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V22" s="36"/>
+      <x:c r="X22" s="36"/>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
       <x:c r="A23" s="36"/>
@@ -1523,13 +1577,15 @@
       <x:c r="Q23" s="36"/>
       <x:c r="R23" s="36"/>
       <x:c r="S23" s="36"/>
-      <x:c r="T23" s="38" t="str">
+      <x:c r="T23" s="36"/>
+      <x:c r="U23" s="36"/>
+      <x:c r="V23" s="38" t="str">
         <x:f>IF(B23="","","https://hlctex.com/textile/products/"&amp;B23&amp;"/")</x:f>
       </x:c>
-      <x:c r="U23" s="38" t="str">
+      <x:c r="W23" s="38" t="str">
         <x:f>IF(B23="","",IF(A23&lt;&gt;"YES","未发布",IF(OR(C23="",D23="",J23=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V23" s="36"/>
+      <x:c r="X23" s="36"/>
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
       <x:c r="A24" s="36"/>
@@ -1551,13 +1607,15 @@
       <x:c r="Q24" s="36"/>
       <x:c r="R24" s="36"/>
       <x:c r="S24" s="36"/>
-      <x:c r="T24" s="38" t="str">
+      <x:c r="T24" s="36"/>
+      <x:c r="U24" s="36"/>
+      <x:c r="V24" s="38" t="str">
         <x:f>IF(B24="","","https://hlctex.com/textile/products/"&amp;B24&amp;"/")</x:f>
       </x:c>
-      <x:c r="U24" s="38" t="str">
+      <x:c r="W24" s="38" t="str">
         <x:f>IF(B24="","",IF(A24&lt;&gt;"YES","未发布",IF(OR(C24="",D24="",J24=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V24" s="36"/>
+      <x:c r="X24" s="36"/>
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
       <x:c r="A25" s="36"/>
@@ -1579,13 +1637,15 @@
       <x:c r="Q25" s="36"/>
       <x:c r="R25" s="36"/>
       <x:c r="S25" s="36"/>
-      <x:c r="T25" s="38" t="str">
+      <x:c r="T25" s="36"/>
+      <x:c r="U25" s="36"/>
+      <x:c r="V25" s="38" t="str">
         <x:f>IF(B25="","","https://hlctex.com/textile/products/"&amp;B25&amp;"/")</x:f>
       </x:c>
-      <x:c r="U25" s="38" t="str">
+      <x:c r="W25" s="38" t="str">
         <x:f>IF(B25="","",IF(A25&lt;&gt;"YES","未发布",IF(OR(C25="",D25="",J25=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V25" s="36"/>
+      <x:c r="X25" s="36"/>
     </x:row>
     <x:row r="26" ht="42" customHeight="1">
       <x:c r="A26" s="36"/>
@@ -1607,13 +1667,15 @@
       <x:c r="Q26" s="36"/>
       <x:c r="R26" s="36"/>
       <x:c r="S26" s="36"/>
-      <x:c r="T26" s="38" t="str">
+      <x:c r="T26" s="36"/>
+      <x:c r="U26" s="36"/>
+      <x:c r="V26" s="38" t="str">
         <x:f>IF(B26="","","https://hlctex.com/textile/products/"&amp;B26&amp;"/")</x:f>
       </x:c>
-      <x:c r="U26" s="38" t="str">
+      <x:c r="W26" s="38" t="str">
         <x:f>IF(B26="","",IF(A26&lt;&gt;"YES","未发布",IF(OR(C26="",D26="",J26=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V26" s="36"/>
+      <x:c r="X26" s="36"/>
     </x:row>
     <x:row r="27" ht="42" customHeight="1">
       <x:c r="A27" s="36"/>
@@ -1635,13 +1697,15 @@
       <x:c r="Q27" s="36"/>
       <x:c r="R27" s="36"/>
       <x:c r="S27" s="36"/>
-      <x:c r="T27" s="38" t="str">
+      <x:c r="T27" s="36"/>
+      <x:c r="U27" s="36"/>
+      <x:c r="V27" s="38" t="str">
         <x:f>IF(B27="","","https://hlctex.com/textile/products/"&amp;B27&amp;"/")</x:f>
       </x:c>
-      <x:c r="U27" s="38" t="str">
+      <x:c r="W27" s="38" t="str">
         <x:f>IF(B27="","",IF(A27&lt;&gt;"YES","未发布",IF(OR(C27="",D27="",J27=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V27" s="36"/>
+      <x:c r="X27" s="36"/>
     </x:row>
     <x:row r="28" ht="42" customHeight="1">
       <x:c r="A28" s="36"/>
@@ -1663,13 +1727,15 @@
       <x:c r="Q28" s="36"/>
       <x:c r="R28" s="36"/>
       <x:c r="S28" s="36"/>
-      <x:c r="T28" s="38" t="str">
+      <x:c r="T28" s="36"/>
+      <x:c r="U28" s="36"/>
+      <x:c r="V28" s="38" t="str">
         <x:f>IF(B28="","","https://hlctex.com/textile/products/"&amp;B28&amp;"/")</x:f>
       </x:c>
-      <x:c r="U28" s="38" t="str">
+      <x:c r="W28" s="38" t="str">
         <x:f>IF(B28="","",IF(A28&lt;&gt;"YES","未发布",IF(OR(C28="",D28="",J28=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V28" s="36"/>
+      <x:c r="X28" s="36"/>
     </x:row>
     <x:row r="29" ht="42" customHeight="1">
       <x:c r="A29" s="36"/>
@@ -1691,13 +1757,15 @@
       <x:c r="Q29" s="36"/>
       <x:c r="R29" s="36"/>
       <x:c r="S29" s="36"/>
-      <x:c r="T29" s="38" t="str">
+      <x:c r="T29" s="36"/>
+      <x:c r="U29" s="36"/>
+      <x:c r="V29" s="38" t="str">
         <x:f>IF(B29="","","https://hlctex.com/textile/products/"&amp;B29&amp;"/")</x:f>
       </x:c>
-      <x:c r="U29" s="38" t="str">
+      <x:c r="W29" s="38" t="str">
         <x:f>IF(B29="","",IF(A29&lt;&gt;"YES","未发布",IF(OR(C29="",D29="",J29=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V29" s="36"/>
+      <x:c r="X29" s="36"/>
     </x:row>
     <x:row r="30" ht="42" customHeight="1">
       <x:c r="A30" s="36"/>
@@ -1719,13 +1787,15 @@
       <x:c r="Q30" s="36"/>
       <x:c r="R30" s="36"/>
       <x:c r="S30" s="36"/>
-      <x:c r="T30" s="38" t="str">
+      <x:c r="T30" s="36"/>
+      <x:c r="U30" s="36"/>
+      <x:c r="V30" s="38" t="str">
         <x:f>IF(B30="","","https://hlctex.com/textile/products/"&amp;B30&amp;"/")</x:f>
       </x:c>
-      <x:c r="U30" s="38" t="str">
+      <x:c r="W30" s="38" t="str">
         <x:f>IF(B30="","",IF(A30&lt;&gt;"YES","未发布",IF(OR(C30="",D30="",J30=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V30" s="36"/>
+      <x:c r="X30" s="36"/>
     </x:row>
     <x:row r="31" ht="42" customHeight="1">
       <x:c r="A31" s="36"/>
@@ -1747,13 +1817,15 @@
       <x:c r="Q31" s="36"/>
       <x:c r="R31" s="36"/>
       <x:c r="S31" s="36"/>
-      <x:c r="T31" s="38" t="str">
+      <x:c r="T31" s="36"/>
+      <x:c r="U31" s="36"/>
+      <x:c r="V31" s="38" t="str">
         <x:f>IF(B31="","","https://hlctex.com/textile/products/"&amp;B31&amp;"/")</x:f>
       </x:c>
-      <x:c r="U31" s="38" t="str">
+      <x:c r="W31" s="38" t="str">
         <x:f>IF(B31="","",IF(A31&lt;&gt;"YES","未发布",IF(OR(C31="",D31="",J31=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V31" s="36"/>
+      <x:c r="X31" s="36"/>
     </x:row>
     <x:row r="32" ht="42" customHeight="1">
       <x:c r="A32" s="36"/>
@@ -1775,13 +1847,15 @@
       <x:c r="Q32" s="36"/>
       <x:c r="R32" s="36"/>
       <x:c r="S32" s="36"/>
-      <x:c r="T32" s="38" t="str">
+      <x:c r="T32" s="36"/>
+      <x:c r="U32" s="36"/>
+      <x:c r="V32" s="38" t="str">
         <x:f>IF(B32="","","https://hlctex.com/textile/products/"&amp;B32&amp;"/")</x:f>
       </x:c>
-      <x:c r="U32" s="38" t="str">
+      <x:c r="W32" s="38" t="str">
         <x:f>IF(B32="","",IF(A32&lt;&gt;"YES","未发布",IF(OR(C32="",D32="",J32=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V32" s="36"/>
+      <x:c r="X32" s="36"/>
     </x:row>
     <x:row r="33" ht="42" customHeight="1">
       <x:c r="A33" s="36"/>
@@ -1803,13 +1877,15 @@
       <x:c r="Q33" s="36"/>
       <x:c r="R33" s="36"/>
       <x:c r="S33" s="36"/>
-      <x:c r="T33" s="38" t="str">
+      <x:c r="T33" s="36"/>
+      <x:c r="U33" s="36"/>
+      <x:c r="V33" s="38" t="str">
         <x:f>IF(B33="","","https://hlctex.com/textile/products/"&amp;B33&amp;"/")</x:f>
       </x:c>
-      <x:c r="U33" s="38" t="str">
+      <x:c r="W33" s="38" t="str">
         <x:f>IF(B33="","",IF(A33&lt;&gt;"YES","未发布",IF(OR(C33="",D33="",J33=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V33" s="36"/>
+      <x:c r="X33" s="36"/>
     </x:row>
     <x:row r="34" ht="42" customHeight="1">
       <x:c r="A34" s="36"/>
@@ -1831,13 +1907,15 @@
       <x:c r="Q34" s="36"/>
       <x:c r="R34" s="36"/>
       <x:c r="S34" s="36"/>
-      <x:c r="T34" s="38" t="str">
+      <x:c r="T34" s="36"/>
+      <x:c r="U34" s="36"/>
+      <x:c r="V34" s="38" t="str">
         <x:f>IF(B34="","","https://hlctex.com/textile/products/"&amp;B34&amp;"/")</x:f>
       </x:c>
-      <x:c r="U34" s="38" t="str">
+      <x:c r="W34" s="38" t="str">
         <x:f>IF(B34="","",IF(A34&lt;&gt;"YES","未发布",IF(OR(C34="",D34="",J34=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V34" s="36"/>
+      <x:c r="X34" s="36"/>
     </x:row>
     <x:row r="35" ht="42" customHeight="1">
       <x:c r="A35" s="36"/>
@@ -1859,13 +1937,15 @@
       <x:c r="Q35" s="36"/>
       <x:c r="R35" s="36"/>
       <x:c r="S35" s="36"/>
-      <x:c r="T35" s="38" t="str">
+      <x:c r="T35" s="36"/>
+      <x:c r="U35" s="36"/>
+      <x:c r="V35" s="38" t="str">
         <x:f>IF(B35="","","https://hlctex.com/textile/products/"&amp;B35&amp;"/")</x:f>
       </x:c>
-      <x:c r="U35" s="38" t="str">
+      <x:c r="W35" s="38" t="str">
         <x:f>IF(B35="","",IF(A35&lt;&gt;"YES","未发布",IF(OR(C35="",D35="",J35=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V35" s="36"/>
+      <x:c r="X35" s="36"/>
     </x:row>
     <x:row r="36" ht="42" customHeight="1">
       <x:c r="A36" s="36"/>
@@ -1887,13 +1967,15 @@
       <x:c r="Q36" s="36"/>
       <x:c r="R36" s="36"/>
       <x:c r="S36" s="36"/>
-      <x:c r="T36" s="38" t="str">
+      <x:c r="T36" s="36"/>
+      <x:c r="U36" s="36"/>
+      <x:c r="V36" s="38" t="str">
         <x:f>IF(B36="","","https://hlctex.com/textile/products/"&amp;B36&amp;"/")</x:f>
       </x:c>
-      <x:c r="U36" s="38" t="str">
+      <x:c r="W36" s="38" t="str">
         <x:f>IF(B36="","",IF(A36&lt;&gt;"YES","未发布",IF(OR(C36="",D36="",J36=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V36" s="36"/>
+      <x:c r="X36" s="36"/>
     </x:row>
     <x:row r="37" ht="42" customHeight="1">
       <x:c r="A37" s="36"/>
@@ -1915,13 +1997,15 @@
       <x:c r="Q37" s="36"/>
       <x:c r="R37" s="36"/>
       <x:c r="S37" s="36"/>
-      <x:c r="T37" s="38" t="str">
+      <x:c r="T37" s="36"/>
+      <x:c r="U37" s="36"/>
+      <x:c r="V37" s="38" t="str">
         <x:f>IF(B37="","","https://hlctex.com/textile/products/"&amp;B37&amp;"/")</x:f>
       </x:c>
-      <x:c r="U37" s="38" t="str">
+      <x:c r="W37" s="38" t="str">
         <x:f>IF(B37="","",IF(A37&lt;&gt;"YES","未发布",IF(OR(C37="",D37="",J37=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V37" s="36"/>
+      <x:c r="X37" s="36"/>
     </x:row>
     <x:row r="38" ht="42" customHeight="1">
       <x:c r="A38" s="36"/>
@@ -1943,13 +2027,15 @@
       <x:c r="Q38" s="36"/>
       <x:c r="R38" s="36"/>
       <x:c r="S38" s="36"/>
-      <x:c r="T38" s="38" t="str">
+      <x:c r="T38" s="36"/>
+      <x:c r="U38" s="36"/>
+      <x:c r="V38" s="38" t="str">
         <x:f>IF(B38="","","https://hlctex.com/textile/products/"&amp;B38&amp;"/")</x:f>
       </x:c>
-      <x:c r="U38" s="38" t="str">
+      <x:c r="W38" s="38" t="str">
         <x:f>IF(B38="","",IF(A38&lt;&gt;"YES","未发布",IF(OR(C38="",D38="",J38=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V38" s="36"/>
+      <x:c r="X38" s="36"/>
     </x:row>
     <x:row r="39" ht="42" customHeight="1">
       <x:c r="A39" s="36"/>
@@ -1971,13 +2057,15 @@
       <x:c r="Q39" s="36"/>
       <x:c r="R39" s="36"/>
       <x:c r="S39" s="36"/>
-      <x:c r="T39" s="38" t="str">
+      <x:c r="T39" s="36"/>
+      <x:c r="U39" s="36"/>
+      <x:c r="V39" s="38" t="str">
         <x:f>IF(B39="","","https://hlctex.com/textile/products/"&amp;B39&amp;"/")</x:f>
       </x:c>
-      <x:c r="U39" s="38" t="str">
+      <x:c r="W39" s="38" t="str">
         <x:f>IF(B39="","",IF(A39&lt;&gt;"YES","未发布",IF(OR(C39="",D39="",J39=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V39" s="36"/>
+      <x:c r="X39" s="36"/>
     </x:row>
     <x:row r="40" ht="42" customHeight="1">
       <x:c r="A40" s="36"/>
@@ -1999,13 +2087,15 @@
       <x:c r="Q40" s="36"/>
       <x:c r="R40" s="36"/>
       <x:c r="S40" s="36"/>
-      <x:c r="T40" s="38" t="str">
+      <x:c r="T40" s="36"/>
+      <x:c r="U40" s="36"/>
+      <x:c r="V40" s="38" t="str">
         <x:f>IF(B40="","","https://hlctex.com/textile/products/"&amp;B40&amp;"/")</x:f>
       </x:c>
-      <x:c r="U40" s="38" t="str">
+      <x:c r="W40" s="38" t="str">
         <x:f>IF(B40="","",IF(A40&lt;&gt;"YES","未发布",IF(OR(C40="",D40="",J40=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V40" s="36"/>
+      <x:c r="X40" s="36"/>
     </x:row>
     <x:row r="41" ht="42" customHeight="1">
       <x:c r="A41" s="36"/>
@@ -2027,13 +2117,15 @@
       <x:c r="Q41" s="36"/>
       <x:c r="R41" s="36"/>
       <x:c r="S41" s="36"/>
-      <x:c r="T41" s="38" t="str">
+      <x:c r="T41" s="36"/>
+      <x:c r="U41" s="36"/>
+      <x:c r="V41" s="38" t="str">
         <x:f>IF(B41="","","https://hlctex.com/textile/products/"&amp;B41&amp;"/")</x:f>
       </x:c>
-      <x:c r="U41" s="38" t="str">
+      <x:c r="W41" s="38" t="str">
         <x:f>IF(B41="","",IF(A41&lt;&gt;"YES","未发布",IF(OR(C41="",D41="",J41=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V41" s="36"/>
+      <x:c r="X41" s="36"/>
     </x:row>
     <x:row r="42" ht="42" customHeight="1">
       <x:c r="A42" s="36"/>
@@ -2055,13 +2147,15 @@
       <x:c r="Q42" s="36"/>
       <x:c r="R42" s="36"/>
       <x:c r="S42" s="36"/>
-      <x:c r="T42" s="38" t="str">
+      <x:c r="T42" s="36"/>
+      <x:c r="U42" s="36"/>
+      <x:c r="V42" s="38" t="str">
         <x:f>IF(B42="","","https://hlctex.com/textile/products/"&amp;B42&amp;"/")</x:f>
       </x:c>
-      <x:c r="U42" s="38" t="str">
+      <x:c r="W42" s="38" t="str">
         <x:f>IF(B42="","",IF(A42&lt;&gt;"YES","未发布",IF(OR(C42="",D42="",J42=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V42" s="36"/>
+      <x:c r="X42" s="36"/>
     </x:row>
     <x:row r="43" ht="42" customHeight="1">
       <x:c r="A43" s="36"/>
@@ -2083,13 +2177,15 @@
       <x:c r="Q43" s="36"/>
       <x:c r="R43" s="36"/>
       <x:c r="S43" s="36"/>
-      <x:c r="T43" s="38" t="str">
+      <x:c r="T43" s="36"/>
+      <x:c r="U43" s="36"/>
+      <x:c r="V43" s="38" t="str">
         <x:f>IF(B43="","","https://hlctex.com/textile/products/"&amp;B43&amp;"/")</x:f>
       </x:c>
-      <x:c r="U43" s="38" t="str">
+      <x:c r="W43" s="38" t="str">
         <x:f>IF(B43="","",IF(A43&lt;&gt;"YES","未发布",IF(OR(C43="",D43="",J43=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V43" s="36"/>
+      <x:c r="X43" s="36"/>
     </x:row>
     <x:row r="44" ht="42" customHeight="1">
       <x:c r="A44" s="36"/>
@@ -2111,13 +2207,15 @@
       <x:c r="Q44" s="36"/>
       <x:c r="R44" s="36"/>
       <x:c r="S44" s="36"/>
-      <x:c r="T44" s="38" t="str">
+      <x:c r="T44" s="36"/>
+      <x:c r="U44" s="36"/>
+      <x:c r="V44" s="38" t="str">
         <x:f>IF(B44="","","https://hlctex.com/textile/products/"&amp;B44&amp;"/")</x:f>
       </x:c>
-      <x:c r="U44" s="38" t="str">
+      <x:c r="W44" s="38" t="str">
         <x:f>IF(B44="","",IF(A44&lt;&gt;"YES","未发布",IF(OR(C44="",D44="",J44=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V44" s="36"/>
+      <x:c r="X44" s="36"/>
     </x:row>
     <x:row r="45" ht="42" customHeight="1">
       <x:c r="A45" s="36"/>
@@ -2139,13 +2237,15 @@
       <x:c r="Q45" s="36"/>
       <x:c r="R45" s="36"/>
       <x:c r="S45" s="36"/>
-      <x:c r="T45" s="38" t="str">
+      <x:c r="T45" s="36"/>
+      <x:c r="U45" s="36"/>
+      <x:c r="V45" s="38" t="str">
         <x:f>IF(B45="","","https://hlctex.com/textile/products/"&amp;B45&amp;"/")</x:f>
       </x:c>
-      <x:c r="U45" s="38" t="str">
+      <x:c r="W45" s="38" t="str">
         <x:f>IF(B45="","",IF(A45&lt;&gt;"YES","未发布",IF(OR(C45="",D45="",J45=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V45" s="36"/>
+      <x:c r="X45" s="36"/>
     </x:row>
     <x:row r="46" ht="42" customHeight="1">
       <x:c r="A46" s="36"/>
@@ -2167,13 +2267,15 @@
       <x:c r="Q46" s="36"/>
       <x:c r="R46" s="36"/>
       <x:c r="S46" s="36"/>
-      <x:c r="T46" s="38" t="str">
+      <x:c r="T46" s="36"/>
+      <x:c r="U46" s="36"/>
+      <x:c r="V46" s="38" t="str">
         <x:f>IF(B46="","","https://hlctex.com/textile/products/"&amp;B46&amp;"/")</x:f>
       </x:c>
-      <x:c r="U46" s="38" t="str">
+      <x:c r="W46" s="38" t="str">
         <x:f>IF(B46="","",IF(A46&lt;&gt;"YES","未发布",IF(OR(C46="",D46="",J46=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V46" s="36"/>
+      <x:c r="X46" s="36"/>
     </x:row>
     <x:row r="47" ht="42" customHeight="1">
       <x:c r="A47" s="36"/>
@@ -2195,13 +2297,15 @@
       <x:c r="Q47" s="36"/>
       <x:c r="R47" s="36"/>
       <x:c r="S47" s="36"/>
-      <x:c r="T47" s="38" t="str">
+      <x:c r="T47" s="36"/>
+      <x:c r="U47" s="36"/>
+      <x:c r="V47" s="38" t="str">
         <x:f>IF(B47="","","https://hlctex.com/textile/products/"&amp;B47&amp;"/")</x:f>
       </x:c>
-      <x:c r="U47" s="38" t="str">
+      <x:c r="W47" s="38" t="str">
         <x:f>IF(B47="","",IF(A47&lt;&gt;"YES","未发布",IF(OR(C47="",D47="",J47=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V47" s="36"/>
+      <x:c r="X47" s="36"/>
     </x:row>
     <x:row r="48" ht="42" customHeight="1">
       <x:c r="A48" s="36"/>
@@ -2223,13 +2327,15 @@
       <x:c r="Q48" s="36"/>
       <x:c r="R48" s="36"/>
       <x:c r="S48" s="36"/>
-      <x:c r="T48" s="38" t="str">
+      <x:c r="T48" s="36"/>
+      <x:c r="U48" s="36"/>
+      <x:c r="V48" s="38" t="str">
         <x:f>IF(B48="","","https://hlctex.com/textile/products/"&amp;B48&amp;"/")</x:f>
       </x:c>
-      <x:c r="U48" s="38" t="str">
+      <x:c r="W48" s="38" t="str">
         <x:f>IF(B48="","",IF(A48&lt;&gt;"YES","未发布",IF(OR(C48="",D48="",J48=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V48" s="36"/>
+      <x:c r="X48" s="36"/>
     </x:row>
     <x:row r="49" ht="42" customHeight="1">
       <x:c r="A49" s="36"/>
@@ -2251,13 +2357,15 @@
       <x:c r="Q49" s="36"/>
       <x:c r="R49" s="36"/>
       <x:c r="S49" s="36"/>
-      <x:c r="T49" s="38" t="str">
+      <x:c r="T49" s="36"/>
+      <x:c r="U49" s="36"/>
+      <x:c r="V49" s="38" t="str">
         <x:f>IF(B49="","","https://hlctex.com/textile/products/"&amp;B49&amp;"/")</x:f>
       </x:c>
-      <x:c r="U49" s="38" t="str">
+      <x:c r="W49" s="38" t="str">
         <x:f>IF(B49="","",IF(A49&lt;&gt;"YES","未发布",IF(OR(C49="",D49="",J49=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V49" s="36"/>
+      <x:c r="X49" s="36"/>
     </x:row>
     <x:row r="50" ht="42" customHeight="1">
       <x:c r="A50" s="36"/>
@@ -2279,13 +2387,15 @@
       <x:c r="Q50" s="36"/>
       <x:c r="R50" s="36"/>
       <x:c r="S50" s="36"/>
-      <x:c r="T50" s="38" t="str">
+      <x:c r="T50" s="36"/>
+      <x:c r="U50" s="36"/>
+      <x:c r="V50" s="38" t="str">
         <x:f>IF(B50="","","https://hlctex.com/textile/products/"&amp;B50&amp;"/")</x:f>
       </x:c>
-      <x:c r="U50" s="38" t="str">
+      <x:c r="W50" s="38" t="str">
         <x:f>IF(B50="","",IF(A50&lt;&gt;"YES","未发布",IF(OR(C50="",D50="",J50=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V50" s="36"/>
+      <x:c r="X50" s="36"/>
     </x:row>
     <x:row r="51" ht="42" customHeight="1">
       <x:c r="A51" s="36"/>
@@ -2307,13 +2417,15 @@
       <x:c r="Q51" s="36"/>
       <x:c r="R51" s="36"/>
       <x:c r="S51" s="36"/>
-      <x:c r="T51" s="38" t="str">
+      <x:c r="T51" s="36"/>
+      <x:c r="U51" s="36"/>
+      <x:c r="V51" s="38" t="str">
         <x:f>IF(B51="","","https://hlctex.com/textile/products/"&amp;B51&amp;"/")</x:f>
       </x:c>
-      <x:c r="U51" s="38" t="str">
+      <x:c r="W51" s="38" t="str">
         <x:f>IF(B51="","",IF(A51&lt;&gt;"YES","未发布",IF(OR(C51="",D51="",J51=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V51" s="36"/>
+      <x:c r="X51" s="36"/>
     </x:row>
     <x:row r="52" ht="42" customHeight="1">
       <x:c r="A52" s="36"/>
@@ -2335,13 +2447,15 @@
       <x:c r="Q52" s="36"/>
       <x:c r="R52" s="36"/>
       <x:c r="S52" s="36"/>
-      <x:c r="T52" s="38" t="str">
+      <x:c r="T52" s="36"/>
+      <x:c r="U52" s="36"/>
+      <x:c r="V52" s="38" t="str">
         <x:f>IF(B52="","","https://hlctex.com/textile/products/"&amp;B52&amp;"/")</x:f>
       </x:c>
-      <x:c r="U52" s="38" t="str">
+      <x:c r="W52" s="38" t="str">
         <x:f>IF(B52="","",IF(A52&lt;&gt;"YES","未发布",IF(OR(C52="",D52="",J52=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V52" s="36"/>
+      <x:c r="X52" s="36"/>
     </x:row>
     <x:row r="53" ht="42" customHeight="1">
       <x:c r="A53" s="36"/>
@@ -2363,13 +2477,15 @@
       <x:c r="Q53" s="36"/>
       <x:c r="R53" s="36"/>
       <x:c r="S53" s="36"/>
-      <x:c r="T53" s="38" t="str">
+      <x:c r="T53" s="36"/>
+      <x:c r="U53" s="36"/>
+      <x:c r="V53" s="38" t="str">
         <x:f>IF(B53="","","https://hlctex.com/textile/products/"&amp;B53&amp;"/")</x:f>
       </x:c>
-      <x:c r="U53" s="38" t="str">
+      <x:c r="W53" s="38" t="str">
         <x:f>IF(B53="","",IF(A53&lt;&gt;"YES","未发布",IF(OR(C53="",D53="",J53=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V53" s="36"/>
+      <x:c r="X53" s="36"/>
     </x:row>
     <x:row r="54" ht="42" customHeight="1">
       <x:c r="A54" s="36"/>
@@ -2391,13 +2507,15 @@
       <x:c r="Q54" s="36"/>
       <x:c r="R54" s="36"/>
       <x:c r="S54" s="36"/>
-      <x:c r="T54" s="38" t="str">
+      <x:c r="T54" s="36"/>
+      <x:c r="U54" s="36"/>
+      <x:c r="V54" s="38" t="str">
         <x:f>IF(B54="","","https://hlctex.com/textile/products/"&amp;B54&amp;"/")</x:f>
       </x:c>
-      <x:c r="U54" s="38" t="str">
+      <x:c r="W54" s="38" t="str">
         <x:f>IF(B54="","",IF(A54&lt;&gt;"YES","未发布",IF(OR(C54="",D54="",J54=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V54" s="36"/>
+      <x:c r="X54" s="36"/>
     </x:row>
     <x:row r="55" ht="42" customHeight="1">
       <x:c r="A55" s="36"/>
@@ -2419,13 +2537,15 @@
       <x:c r="Q55" s="36"/>
       <x:c r="R55" s="36"/>
       <x:c r="S55" s="36"/>
-      <x:c r="T55" s="38" t="str">
+      <x:c r="T55" s="36"/>
+      <x:c r="U55" s="36"/>
+      <x:c r="V55" s="38" t="str">
         <x:f>IF(B55="","","https://hlctex.com/textile/products/"&amp;B55&amp;"/")</x:f>
       </x:c>
-      <x:c r="U55" s="38" t="str">
+      <x:c r="W55" s="38" t="str">
         <x:f>IF(B55="","",IF(A55&lt;&gt;"YES","未发布",IF(OR(C55="",D55="",J55=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V55" s="36"/>
+      <x:c r="X55" s="36"/>
     </x:row>
     <x:row r="56" ht="42" customHeight="1">
       <x:c r="A56" s="36"/>
@@ -2447,13 +2567,15 @@
       <x:c r="Q56" s="36"/>
       <x:c r="R56" s="36"/>
       <x:c r="S56" s="36"/>
-      <x:c r="T56" s="38" t="str">
+      <x:c r="T56" s="36"/>
+      <x:c r="U56" s="36"/>
+      <x:c r="V56" s="38" t="str">
         <x:f>IF(B56="","","https://hlctex.com/textile/products/"&amp;B56&amp;"/")</x:f>
       </x:c>
-      <x:c r="U56" s="38" t="str">
+      <x:c r="W56" s="38" t="str">
         <x:f>IF(B56="","",IF(A56&lt;&gt;"YES","未发布",IF(OR(C56="",D56="",J56=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V56" s="36"/>
+      <x:c r="X56" s="36"/>
     </x:row>
     <x:row r="57" ht="42" customHeight="1">
       <x:c r="A57" s="36"/>
@@ -2475,13 +2597,15 @@
       <x:c r="Q57" s="36"/>
       <x:c r="R57" s="36"/>
       <x:c r="S57" s="36"/>
-      <x:c r="T57" s="38" t="str">
+      <x:c r="T57" s="36"/>
+      <x:c r="U57" s="36"/>
+      <x:c r="V57" s="38" t="str">
         <x:f>IF(B57="","","https://hlctex.com/textile/products/"&amp;B57&amp;"/")</x:f>
       </x:c>
-      <x:c r="U57" s="38" t="str">
+      <x:c r="W57" s="38" t="str">
         <x:f>IF(B57="","",IF(A57&lt;&gt;"YES","未发布",IF(OR(C57="",D57="",J57=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V57" s="36"/>
+      <x:c r="X57" s="36"/>
     </x:row>
     <x:row r="58" ht="42" customHeight="1">
       <x:c r="A58" s="36"/>
@@ -2503,13 +2627,15 @@
       <x:c r="Q58" s="36"/>
       <x:c r="R58" s="36"/>
       <x:c r="S58" s="36"/>
-      <x:c r="T58" s="38" t="str">
+      <x:c r="T58" s="36"/>
+      <x:c r="U58" s="36"/>
+      <x:c r="V58" s="38" t="str">
         <x:f>IF(B58="","","https://hlctex.com/textile/products/"&amp;B58&amp;"/")</x:f>
       </x:c>
-      <x:c r="U58" s="38" t="str">
+      <x:c r="W58" s="38" t="str">
         <x:f>IF(B58="","",IF(A58&lt;&gt;"YES","未发布",IF(OR(C58="",D58="",J58=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V58" s="36"/>
+      <x:c r="X58" s="36"/>
     </x:row>
     <x:row r="59" ht="42" customHeight="1">
       <x:c r="A59" s="36"/>
@@ -2531,13 +2657,15 @@
       <x:c r="Q59" s="36"/>
       <x:c r="R59" s="36"/>
       <x:c r="S59" s="36"/>
-      <x:c r="T59" s="38" t="str">
+      <x:c r="T59" s="36"/>
+      <x:c r="U59" s="36"/>
+      <x:c r="V59" s="38" t="str">
         <x:f>IF(B59="","","https://hlctex.com/textile/products/"&amp;B59&amp;"/")</x:f>
       </x:c>
-      <x:c r="U59" s="38" t="str">
+      <x:c r="W59" s="38" t="str">
         <x:f>IF(B59="","",IF(A59&lt;&gt;"YES","未发布",IF(OR(C59="",D59="",J59=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V59" s="36"/>
+      <x:c r="X59" s="36"/>
     </x:row>
     <x:row r="60" ht="42" customHeight="1">
       <x:c r="A60" s="36"/>
@@ -2559,13 +2687,15 @@
       <x:c r="Q60" s="36"/>
       <x:c r="R60" s="36"/>
       <x:c r="S60" s="36"/>
-      <x:c r="T60" s="38" t="str">
+      <x:c r="T60" s="36"/>
+      <x:c r="U60" s="36"/>
+      <x:c r="V60" s="38" t="str">
         <x:f>IF(B60="","","https://hlctex.com/textile/products/"&amp;B60&amp;"/")</x:f>
       </x:c>
-      <x:c r="U60" s="38" t="str">
+      <x:c r="W60" s="38" t="str">
         <x:f>IF(B60="","",IF(A60&lt;&gt;"YES","未发布",IF(OR(C60="",D60="",J60=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V60" s="36"/>
+      <x:c r="X60" s="36"/>
     </x:row>
     <x:row r="61" ht="42" customHeight="1">
       <x:c r="A61" s="36"/>
@@ -2587,13 +2717,15 @@
       <x:c r="Q61" s="36"/>
       <x:c r="R61" s="36"/>
       <x:c r="S61" s="36"/>
-      <x:c r="T61" s="38" t="str">
+      <x:c r="T61" s="36"/>
+      <x:c r="U61" s="36"/>
+      <x:c r="V61" s="38" t="str">
         <x:f>IF(B61="","","https://hlctex.com/textile/products/"&amp;B61&amp;"/")</x:f>
       </x:c>
-      <x:c r="U61" s="38" t="str">
+      <x:c r="W61" s="38" t="str">
         <x:f>IF(B61="","",IF(A61&lt;&gt;"YES","未发布",IF(OR(C61="",D61="",J61=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V61" s="36"/>
+      <x:c r="X61" s="36"/>
     </x:row>
     <x:row r="62" ht="42" customHeight="1">
       <x:c r="A62" s="36"/>
@@ -2615,13 +2747,15 @@
       <x:c r="Q62" s="36"/>
       <x:c r="R62" s="36"/>
       <x:c r="S62" s="36"/>
-      <x:c r="T62" s="38" t="str">
+      <x:c r="T62" s="36"/>
+      <x:c r="U62" s="36"/>
+      <x:c r="V62" s="38" t="str">
         <x:f>IF(B62="","","https://hlctex.com/textile/products/"&amp;B62&amp;"/")</x:f>
       </x:c>
-      <x:c r="U62" s="38" t="str">
+      <x:c r="W62" s="38" t="str">
         <x:f>IF(B62="","",IF(A62&lt;&gt;"YES","未发布",IF(OR(C62="",D62="",J62=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V62" s="36"/>
+      <x:c r="X62" s="36"/>
     </x:row>
     <x:row r="63" ht="42" customHeight="1">
       <x:c r="A63" s="36"/>
@@ -2643,13 +2777,15 @@
       <x:c r="Q63" s="36"/>
       <x:c r="R63" s="36"/>
       <x:c r="S63" s="36"/>
-      <x:c r="T63" s="38" t="str">
+      <x:c r="T63" s="36"/>
+      <x:c r="U63" s="36"/>
+      <x:c r="V63" s="38" t="str">
         <x:f>IF(B63="","","https://hlctex.com/textile/products/"&amp;B63&amp;"/")</x:f>
       </x:c>
-      <x:c r="U63" s="38" t="str">
+      <x:c r="W63" s="38" t="str">
         <x:f>IF(B63="","",IF(A63&lt;&gt;"YES","未发布",IF(OR(C63="",D63="",J63=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V63" s="36"/>
+      <x:c r="X63" s="36"/>
     </x:row>
     <x:row r="64" ht="42" customHeight="1">
       <x:c r="A64" s="36"/>
@@ -2671,13 +2807,15 @@
       <x:c r="Q64" s="36"/>
       <x:c r="R64" s="36"/>
       <x:c r="S64" s="36"/>
-      <x:c r="T64" s="38" t="str">
+      <x:c r="T64" s="36"/>
+      <x:c r="U64" s="36"/>
+      <x:c r="V64" s="38" t="str">
         <x:f>IF(B64="","","https://hlctex.com/textile/products/"&amp;B64&amp;"/")</x:f>
       </x:c>
-      <x:c r="U64" s="38" t="str">
+      <x:c r="W64" s="38" t="str">
         <x:f>IF(B64="","",IF(A64&lt;&gt;"YES","未发布",IF(OR(C64="",D64="",J64=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V64" s="36"/>
+      <x:c r="X64" s="36"/>
     </x:row>
     <x:row r="65" ht="42" customHeight="1">
       <x:c r="A65" s="36"/>
@@ -2699,13 +2837,15 @@
       <x:c r="Q65" s="36"/>
       <x:c r="R65" s="36"/>
       <x:c r="S65" s="36"/>
-      <x:c r="T65" s="38" t="str">
+      <x:c r="T65" s="36"/>
+      <x:c r="U65" s="36"/>
+      <x:c r="V65" s="38" t="str">
         <x:f>IF(B65="","","https://hlctex.com/textile/products/"&amp;B65&amp;"/")</x:f>
       </x:c>
-      <x:c r="U65" s="38" t="str">
+      <x:c r="W65" s="38" t="str">
         <x:f>IF(B65="","",IF(A65&lt;&gt;"YES","未发布",IF(OR(C65="",D65="",J65=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V65" s="36"/>
+      <x:c r="X65" s="36"/>
     </x:row>
     <x:row r="66" ht="42" customHeight="1">
       <x:c r="A66" s="36"/>
@@ -2727,13 +2867,15 @@
       <x:c r="Q66" s="36"/>
       <x:c r="R66" s="36"/>
       <x:c r="S66" s="36"/>
-      <x:c r="T66" s="38" t="str">
+      <x:c r="T66" s="36"/>
+      <x:c r="U66" s="36"/>
+      <x:c r="V66" s="38" t="str">
         <x:f>IF(B66="","","https://hlctex.com/textile/products/"&amp;B66&amp;"/")</x:f>
       </x:c>
-      <x:c r="U66" s="38" t="str">
+      <x:c r="W66" s="38" t="str">
         <x:f>IF(B66="","",IF(A66&lt;&gt;"YES","未发布",IF(OR(C66="",D66="",J66=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V66" s="36"/>
+      <x:c r="X66" s="36"/>
     </x:row>
     <x:row r="67" ht="42" customHeight="1">
       <x:c r="A67" s="36"/>
@@ -2755,13 +2897,15 @@
       <x:c r="Q67" s="36"/>
       <x:c r="R67" s="36"/>
       <x:c r="S67" s="36"/>
-      <x:c r="T67" s="38" t="str">
+      <x:c r="T67" s="36"/>
+      <x:c r="U67" s="36"/>
+      <x:c r="V67" s="38" t="str">
         <x:f>IF(B67="","","https://hlctex.com/textile/products/"&amp;B67&amp;"/")</x:f>
       </x:c>
-      <x:c r="U67" s="38" t="str">
+      <x:c r="W67" s="38" t="str">
         <x:f>IF(B67="","",IF(A67&lt;&gt;"YES","未发布",IF(OR(C67="",D67="",J67=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V67" s="36"/>
+      <x:c r="X67" s="36"/>
     </x:row>
     <x:row r="68" ht="42" customHeight="1">
       <x:c r="A68" s="36"/>
@@ -2783,13 +2927,15 @@
       <x:c r="Q68" s="36"/>
       <x:c r="R68" s="36"/>
       <x:c r="S68" s="36"/>
-      <x:c r="T68" s="38" t="str">
+      <x:c r="T68" s="36"/>
+      <x:c r="U68" s="36"/>
+      <x:c r="V68" s="38" t="str">
         <x:f>IF(B68="","","https://hlctex.com/textile/products/"&amp;B68&amp;"/")</x:f>
       </x:c>
-      <x:c r="U68" s="38" t="str">
+      <x:c r="W68" s="38" t="str">
         <x:f>IF(B68="","",IF(A68&lt;&gt;"YES","未发布",IF(OR(C68="",D68="",J68=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V68" s="36"/>
+      <x:c r="X68" s="36"/>
     </x:row>
     <x:row r="69" ht="42" customHeight="1">
       <x:c r="A69" s="36"/>
@@ -2811,13 +2957,15 @@
       <x:c r="Q69" s="36"/>
       <x:c r="R69" s="36"/>
       <x:c r="S69" s="36"/>
-      <x:c r="T69" s="38" t="str">
+      <x:c r="T69" s="36"/>
+      <x:c r="U69" s="36"/>
+      <x:c r="V69" s="38" t="str">
         <x:f>IF(B69="","","https://hlctex.com/textile/products/"&amp;B69&amp;"/")</x:f>
       </x:c>
-      <x:c r="U69" s="38" t="str">
+      <x:c r="W69" s="38" t="str">
         <x:f>IF(B69="","",IF(A69&lt;&gt;"YES","未发布",IF(OR(C69="",D69="",J69=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V69" s="36"/>
+      <x:c r="X69" s="36"/>
     </x:row>
     <x:row r="70" ht="42" customHeight="1">
       <x:c r="A70" s="36"/>
@@ -2839,13 +2987,15 @@
       <x:c r="Q70" s="36"/>
       <x:c r="R70" s="36"/>
       <x:c r="S70" s="36"/>
-      <x:c r="T70" s="38" t="str">
+      <x:c r="T70" s="36"/>
+      <x:c r="U70" s="36"/>
+      <x:c r="V70" s="38" t="str">
         <x:f>IF(B70="","","https://hlctex.com/textile/products/"&amp;B70&amp;"/")</x:f>
       </x:c>
-      <x:c r="U70" s="38" t="str">
+      <x:c r="W70" s="38" t="str">
         <x:f>IF(B70="","",IF(A70&lt;&gt;"YES","未发布",IF(OR(C70="",D70="",J70=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V70" s="36"/>
+      <x:c r="X70" s="36"/>
     </x:row>
     <x:row r="71" ht="42" customHeight="1">
       <x:c r="A71" s="36"/>
@@ -2867,13 +3017,15 @@
       <x:c r="Q71" s="36"/>
       <x:c r="R71" s="36"/>
       <x:c r="S71" s="36"/>
-      <x:c r="T71" s="38" t="str">
+      <x:c r="T71" s="36"/>
+      <x:c r="U71" s="36"/>
+      <x:c r="V71" s="38" t="str">
         <x:f>IF(B71="","","https://hlctex.com/textile/products/"&amp;B71&amp;"/")</x:f>
       </x:c>
-      <x:c r="U71" s="38" t="str">
+      <x:c r="W71" s="38" t="str">
         <x:f>IF(B71="","",IF(A71&lt;&gt;"YES","未发布",IF(OR(C71="",D71="",J71=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V71" s="36"/>
+      <x:c r="X71" s="36"/>
     </x:row>
     <x:row r="72" ht="42" customHeight="1">
       <x:c r="A72" s="36"/>
@@ -2895,13 +3047,15 @@
       <x:c r="Q72" s="36"/>
       <x:c r="R72" s="36"/>
       <x:c r="S72" s="36"/>
-      <x:c r="T72" s="38" t="str">
+      <x:c r="T72" s="36"/>
+      <x:c r="U72" s="36"/>
+      <x:c r="V72" s="38" t="str">
         <x:f>IF(B72="","","https://hlctex.com/textile/products/"&amp;B72&amp;"/")</x:f>
       </x:c>
-      <x:c r="U72" s="38" t="str">
+      <x:c r="W72" s="38" t="str">
         <x:f>IF(B72="","",IF(A72&lt;&gt;"YES","未发布",IF(OR(C72="",D72="",J72=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V72" s="36"/>
+      <x:c r="X72" s="36"/>
     </x:row>
     <x:row r="73" ht="42" customHeight="1">
       <x:c r="A73" s="36"/>
@@ -2923,13 +3077,15 @@
       <x:c r="Q73" s="36"/>
       <x:c r="R73" s="36"/>
       <x:c r="S73" s="36"/>
-      <x:c r="T73" s="38" t="str">
+      <x:c r="T73" s="36"/>
+      <x:c r="U73" s="36"/>
+      <x:c r="V73" s="38" t="str">
         <x:f>IF(B73="","","https://hlctex.com/textile/products/"&amp;B73&amp;"/")</x:f>
       </x:c>
-      <x:c r="U73" s="38" t="str">
+      <x:c r="W73" s="38" t="str">
         <x:f>IF(B73="","",IF(A73&lt;&gt;"YES","未发布",IF(OR(C73="",D73="",J73=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V73" s="36"/>
+      <x:c r="X73" s="36"/>
     </x:row>
     <x:row r="74" ht="42" customHeight="1">
       <x:c r="A74" s="36"/>
@@ -2951,13 +3107,15 @@
       <x:c r="Q74" s="36"/>
       <x:c r="R74" s="36"/>
       <x:c r="S74" s="36"/>
-      <x:c r="T74" s="38" t="str">
+      <x:c r="T74" s="36"/>
+      <x:c r="U74" s="36"/>
+      <x:c r="V74" s="38" t="str">
         <x:f>IF(B74="","","https://hlctex.com/textile/products/"&amp;B74&amp;"/")</x:f>
       </x:c>
-      <x:c r="U74" s="38" t="str">
+      <x:c r="W74" s="38" t="str">
         <x:f>IF(B74="","",IF(A74&lt;&gt;"YES","未发布",IF(OR(C74="",D74="",J74=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V74" s="36"/>
+      <x:c r="X74" s="36"/>
     </x:row>
     <x:row r="75" ht="42" customHeight="1">
       <x:c r="A75" s="36"/>
@@ -2979,13 +3137,15 @@
       <x:c r="Q75" s="36"/>
       <x:c r="R75" s="36"/>
       <x:c r="S75" s="36"/>
-      <x:c r="T75" s="38" t="str">
+      <x:c r="T75" s="36"/>
+      <x:c r="U75" s="36"/>
+      <x:c r="V75" s="38" t="str">
         <x:f>IF(B75="","","https://hlctex.com/textile/products/"&amp;B75&amp;"/")</x:f>
       </x:c>
-      <x:c r="U75" s="38" t="str">
+      <x:c r="W75" s="38" t="str">
         <x:f>IF(B75="","",IF(A75&lt;&gt;"YES","未发布",IF(OR(C75="",D75="",J75=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V75" s="36"/>
+      <x:c r="X75" s="36"/>
     </x:row>
     <x:row r="76" ht="42" customHeight="1">
       <x:c r="A76" s="36"/>
@@ -3007,13 +3167,15 @@
       <x:c r="Q76" s="36"/>
       <x:c r="R76" s="36"/>
       <x:c r="S76" s="36"/>
-      <x:c r="T76" s="38" t="str">
+      <x:c r="T76" s="36"/>
+      <x:c r="U76" s="36"/>
+      <x:c r="V76" s="38" t="str">
         <x:f>IF(B76="","","https://hlctex.com/textile/products/"&amp;B76&amp;"/")</x:f>
       </x:c>
-      <x:c r="U76" s="38" t="str">
+      <x:c r="W76" s="38" t="str">
         <x:f>IF(B76="","",IF(A76&lt;&gt;"YES","未发布",IF(OR(C76="",D76="",J76=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V76" s="36"/>
+      <x:c r="X76" s="36"/>
     </x:row>
     <x:row r="77" ht="42" customHeight="1">
       <x:c r="A77" s="36"/>
@@ -3035,13 +3197,15 @@
       <x:c r="Q77" s="36"/>
       <x:c r="R77" s="36"/>
       <x:c r="S77" s="36"/>
-      <x:c r="T77" s="38" t="str">
+      <x:c r="T77" s="36"/>
+      <x:c r="U77" s="36"/>
+      <x:c r="V77" s="38" t="str">
         <x:f>IF(B77="","","https://hlctex.com/textile/products/"&amp;B77&amp;"/")</x:f>
       </x:c>
-      <x:c r="U77" s="38" t="str">
+      <x:c r="W77" s="38" t="str">
         <x:f>IF(B77="","",IF(A77&lt;&gt;"YES","未发布",IF(OR(C77="",D77="",J77=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V77" s="36"/>
+      <x:c r="X77" s="36"/>
     </x:row>
     <x:row r="78" ht="42" customHeight="1">
       <x:c r="A78" s="36"/>
@@ -3063,13 +3227,15 @@
       <x:c r="Q78" s="36"/>
       <x:c r="R78" s="36"/>
       <x:c r="S78" s="36"/>
-      <x:c r="T78" s="38" t="str">
+      <x:c r="T78" s="36"/>
+      <x:c r="U78" s="36"/>
+      <x:c r="V78" s="38" t="str">
         <x:f>IF(B78="","","https://hlctex.com/textile/products/"&amp;B78&amp;"/")</x:f>
       </x:c>
-      <x:c r="U78" s="38" t="str">
+      <x:c r="W78" s="38" t="str">
         <x:f>IF(B78="","",IF(A78&lt;&gt;"YES","未发布",IF(OR(C78="",D78="",J78=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V78" s="36"/>
+      <x:c r="X78" s="36"/>
     </x:row>
     <x:row r="79" ht="42" customHeight="1">
       <x:c r="A79" s="36"/>
@@ -3091,13 +3257,15 @@
       <x:c r="Q79" s="36"/>
       <x:c r="R79" s="36"/>
       <x:c r="S79" s="36"/>
-      <x:c r="T79" s="38" t="str">
+      <x:c r="T79" s="36"/>
+      <x:c r="U79" s="36"/>
+      <x:c r="V79" s="38" t="str">
         <x:f>IF(B79="","","https://hlctex.com/textile/products/"&amp;B79&amp;"/")</x:f>
       </x:c>
-      <x:c r="U79" s="38" t="str">
+      <x:c r="W79" s="38" t="str">
         <x:f>IF(B79="","",IF(A79&lt;&gt;"YES","未发布",IF(OR(C79="",D79="",J79=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V79" s="36"/>
+      <x:c r="X79" s="36"/>
     </x:row>
     <x:row r="80" ht="42" customHeight="1">
       <x:c r="A80" s="36"/>
@@ -3119,13 +3287,15 @@
       <x:c r="Q80" s="36"/>
       <x:c r="R80" s="36"/>
       <x:c r="S80" s="36"/>
-      <x:c r="T80" s="38" t="str">
+      <x:c r="T80" s="36"/>
+      <x:c r="U80" s="36"/>
+      <x:c r="V80" s="38" t="str">
         <x:f>IF(B80="","","https://hlctex.com/textile/products/"&amp;B80&amp;"/")</x:f>
       </x:c>
-      <x:c r="U80" s="38" t="str">
+      <x:c r="W80" s="38" t="str">
         <x:f>IF(B80="","",IF(A80&lt;&gt;"YES","未发布",IF(OR(C80="",D80="",J80=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V80" s="36"/>
+      <x:c r="X80" s="36"/>
     </x:row>
     <x:row r="81" ht="42" customHeight="1">
       <x:c r="A81" s="36"/>
@@ -3147,13 +3317,15 @@
       <x:c r="Q81" s="36"/>
       <x:c r="R81" s="36"/>
       <x:c r="S81" s="36"/>
-      <x:c r="T81" s="38" t="str">
+      <x:c r="T81" s="36"/>
+      <x:c r="U81" s="36"/>
+      <x:c r="V81" s="38" t="str">
         <x:f>IF(B81="","","https://hlctex.com/textile/products/"&amp;B81&amp;"/")</x:f>
       </x:c>
-      <x:c r="U81" s="38" t="str">
+      <x:c r="W81" s="38" t="str">
         <x:f>IF(B81="","",IF(A81&lt;&gt;"YES","未发布",IF(OR(C81="",D81="",J81=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V81" s="36"/>
+      <x:c r="X81" s="36"/>
     </x:row>
     <x:row r="82" ht="42" customHeight="1">
       <x:c r="A82" s="36"/>
@@ -3175,13 +3347,15 @@
       <x:c r="Q82" s="36"/>
       <x:c r="R82" s="36"/>
       <x:c r="S82" s="36"/>
-      <x:c r="T82" s="38" t="str">
+      <x:c r="T82" s="36"/>
+      <x:c r="U82" s="36"/>
+      <x:c r="V82" s="38" t="str">
         <x:f>IF(B82="","","https://hlctex.com/textile/products/"&amp;B82&amp;"/")</x:f>
       </x:c>
-      <x:c r="U82" s="38" t="str">
+      <x:c r="W82" s="38" t="str">
         <x:f>IF(B82="","",IF(A82&lt;&gt;"YES","未发布",IF(OR(C82="",D82="",J82=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V82" s="36"/>
+      <x:c r="X82" s="36"/>
     </x:row>
     <x:row r="83" ht="42" customHeight="1">
       <x:c r="A83" s="36"/>
@@ -3203,13 +3377,15 @@
       <x:c r="Q83" s="36"/>
       <x:c r="R83" s="36"/>
       <x:c r="S83" s="36"/>
-      <x:c r="T83" s="38" t="str">
+      <x:c r="T83" s="36"/>
+      <x:c r="U83" s="36"/>
+      <x:c r="V83" s="38" t="str">
         <x:f>IF(B83="","","https://hlctex.com/textile/products/"&amp;B83&amp;"/")</x:f>
       </x:c>
-      <x:c r="U83" s="38" t="str">
+      <x:c r="W83" s="38" t="str">
         <x:f>IF(B83="","",IF(A83&lt;&gt;"YES","未发布",IF(OR(C83="",D83="",J83=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V83" s="36"/>
+      <x:c r="X83" s="36"/>
     </x:row>
     <x:row r="84" ht="42" customHeight="1">
       <x:c r="A84" s="36"/>
@@ -3231,13 +3407,15 @@
       <x:c r="Q84" s="36"/>
       <x:c r="R84" s="36"/>
       <x:c r="S84" s="36"/>
-      <x:c r="T84" s="38" t="str">
+      <x:c r="T84" s="36"/>
+      <x:c r="U84" s="36"/>
+      <x:c r="V84" s="38" t="str">
         <x:f>IF(B84="","","https://hlctex.com/textile/products/"&amp;B84&amp;"/")</x:f>
       </x:c>
-      <x:c r="U84" s="38" t="str">
+      <x:c r="W84" s="38" t="str">
         <x:f>IF(B84="","",IF(A84&lt;&gt;"YES","未发布",IF(OR(C84="",D84="",J84=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V84" s="36"/>
+      <x:c r="X84" s="36"/>
     </x:row>
     <x:row r="85" ht="42" customHeight="1">
       <x:c r="A85" s="36"/>
@@ -3259,13 +3437,15 @@
       <x:c r="Q85" s="36"/>
       <x:c r="R85" s="36"/>
       <x:c r="S85" s="36"/>
-      <x:c r="T85" s="38" t="str">
+      <x:c r="T85" s="36"/>
+      <x:c r="U85" s="36"/>
+      <x:c r="V85" s="38" t="str">
         <x:f>IF(B85="","","https://hlctex.com/textile/products/"&amp;B85&amp;"/")</x:f>
       </x:c>
-      <x:c r="U85" s="38" t="str">
+      <x:c r="W85" s="38" t="str">
         <x:f>IF(B85="","",IF(A85&lt;&gt;"YES","未发布",IF(OR(C85="",D85="",J85=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V85" s="36"/>
+      <x:c r="X85" s="36"/>
     </x:row>
     <x:row r="86" ht="42" customHeight="1">
       <x:c r="A86" s="36"/>
@@ -3287,13 +3467,15 @@
       <x:c r="Q86" s="36"/>
       <x:c r="R86" s="36"/>
       <x:c r="S86" s="36"/>
-      <x:c r="T86" s="38" t="str">
+      <x:c r="T86" s="36"/>
+      <x:c r="U86" s="36"/>
+      <x:c r="V86" s="38" t="str">
         <x:f>IF(B86="","","https://hlctex.com/textile/products/"&amp;B86&amp;"/")</x:f>
       </x:c>
-      <x:c r="U86" s="38" t="str">
+      <x:c r="W86" s="38" t="str">
         <x:f>IF(B86="","",IF(A86&lt;&gt;"YES","未发布",IF(OR(C86="",D86="",J86=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V86" s="36"/>
+      <x:c r="X86" s="36"/>
     </x:row>
     <x:row r="87" ht="42" customHeight="1">
       <x:c r="A87" s="36"/>
@@ -3315,13 +3497,15 @@
       <x:c r="Q87" s="36"/>
       <x:c r="R87" s="36"/>
       <x:c r="S87" s="36"/>
-      <x:c r="T87" s="38" t="str">
+      <x:c r="T87" s="36"/>
+      <x:c r="U87" s="36"/>
+      <x:c r="V87" s="38" t="str">
         <x:f>IF(B87="","","https://hlctex.com/textile/products/"&amp;B87&amp;"/")</x:f>
       </x:c>
-      <x:c r="U87" s="38" t="str">
+      <x:c r="W87" s="38" t="str">
         <x:f>IF(B87="","",IF(A87&lt;&gt;"YES","未发布",IF(OR(C87="",D87="",J87=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V87" s="36"/>
+      <x:c r="X87" s="36"/>
     </x:row>
     <x:row r="88" ht="42" customHeight="1">
       <x:c r="A88" s="36"/>
@@ -3343,13 +3527,15 @@
       <x:c r="Q88" s="36"/>
       <x:c r="R88" s="36"/>
       <x:c r="S88" s="36"/>
-      <x:c r="T88" s="38" t="str">
+      <x:c r="T88" s="36"/>
+      <x:c r="U88" s="36"/>
+      <x:c r="V88" s="38" t="str">
         <x:f>IF(B88="","","https://hlctex.com/textile/products/"&amp;B88&amp;"/")</x:f>
       </x:c>
-      <x:c r="U88" s="38" t="str">
+      <x:c r="W88" s="38" t="str">
         <x:f>IF(B88="","",IF(A88&lt;&gt;"YES","未发布",IF(OR(C88="",D88="",J88=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V88" s="36"/>
+      <x:c r="X88" s="36"/>
     </x:row>
     <x:row r="89" ht="42" customHeight="1">
       <x:c r="A89" s="36"/>
@@ -3371,13 +3557,15 @@
       <x:c r="Q89" s="36"/>
       <x:c r="R89" s="36"/>
       <x:c r="S89" s="36"/>
-      <x:c r="T89" s="38" t="str">
+      <x:c r="T89" s="36"/>
+      <x:c r="U89" s="36"/>
+      <x:c r="V89" s="38" t="str">
         <x:f>IF(B89="","","https://hlctex.com/textile/products/"&amp;B89&amp;"/")</x:f>
       </x:c>
-      <x:c r="U89" s="38" t="str">
+      <x:c r="W89" s="38" t="str">
         <x:f>IF(B89="","",IF(A89&lt;&gt;"YES","未发布",IF(OR(C89="",D89="",J89=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V89" s="36"/>
+      <x:c r="X89" s="36"/>
     </x:row>
     <x:row r="90" ht="42" customHeight="1">
       <x:c r="A90" s="36"/>
@@ -3399,13 +3587,15 @@
       <x:c r="Q90" s="36"/>
       <x:c r="R90" s="36"/>
       <x:c r="S90" s="36"/>
-      <x:c r="T90" s="38" t="str">
+      <x:c r="T90" s="36"/>
+      <x:c r="U90" s="36"/>
+      <x:c r="V90" s="38" t="str">
         <x:f>IF(B90="","","https://hlctex.com/textile/products/"&amp;B90&amp;"/")</x:f>
       </x:c>
-      <x:c r="U90" s="38" t="str">
+      <x:c r="W90" s="38" t="str">
         <x:f>IF(B90="","",IF(A90&lt;&gt;"YES","未发布",IF(OR(C90="",D90="",J90=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V90" s="36"/>
+      <x:c r="X90" s="36"/>
     </x:row>
     <x:row r="91" ht="42" customHeight="1">
       <x:c r="A91" s="36"/>
@@ -3427,13 +3617,15 @@
       <x:c r="Q91" s="36"/>
       <x:c r="R91" s="36"/>
       <x:c r="S91" s="36"/>
-      <x:c r="T91" s="38" t="str">
+      <x:c r="T91" s="36"/>
+      <x:c r="U91" s="36"/>
+      <x:c r="V91" s="38" t="str">
         <x:f>IF(B91="","","https://hlctex.com/textile/products/"&amp;B91&amp;"/")</x:f>
       </x:c>
-      <x:c r="U91" s="38" t="str">
+      <x:c r="W91" s="38" t="str">
         <x:f>IF(B91="","",IF(A91&lt;&gt;"YES","未发布",IF(OR(C91="",D91="",J91=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V91" s="36"/>
+      <x:c r="X91" s="36"/>
     </x:row>
     <x:row r="92" ht="42" customHeight="1">
       <x:c r="A92" s="36"/>
@@ -3455,13 +3647,15 @@
       <x:c r="Q92" s="36"/>
       <x:c r="R92" s="36"/>
       <x:c r="S92" s="36"/>
-      <x:c r="T92" s="38" t="str">
+      <x:c r="T92" s="36"/>
+      <x:c r="U92" s="36"/>
+      <x:c r="V92" s="38" t="str">
         <x:f>IF(B92="","","https://hlctex.com/textile/products/"&amp;B92&amp;"/")</x:f>
       </x:c>
-      <x:c r="U92" s="38" t="str">
+      <x:c r="W92" s="38" t="str">
         <x:f>IF(B92="","",IF(A92&lt;&gt;"YES","未发布",IF(OR(C92="",D92="",J92=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V92" s="36"/>
+      <x:c r="X92" s="36"/>
     </x:row>
     <x:row r="93" ht="42" customHeight="1">
       <x:c r="A93" s="36"/>
@@ -3483,13 +3677,15 @@
       <x:c r="Q93" s="36"/>
       <x:c r="R93" s="36"/>
       <x:c r="S93" s="36"/>
-      <x:c r="T93" s="38" t="str">
+      <x:c r="T93" s="36"/>
+      <x:c r="U93" s="36"/>
+      <x:c r="V93" s="38" t="str">
         <x:f>IF(B93="","","https://hlctex.com/textile/products/"&amp;B93&amp;"/")</x:f>
       </x:c>
-      <x:c r="U93" s="38" t="str">
+      <x:c r="W93" s="38" t="str">
         <x:f>IF(B93="","",IF(A93&lt;&gt;"YES","未发布",IF(OR(C93="",D93="",J93=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V93" s="36"/>
+      <x:c r="X93" s="36"/>
     </x:row>
     <x:row r="94" ht="42" customHeight="1">
       <x:c r="A94" s="36"/>
@@ -3511,13 +3707,15 @@
       <x:c r="Q94" s="36"/>
       <x:c r="R94" s="36"/>
       <x:c r="S94" s="36"/>
-      <x:c r="T94" s="38" t="str">
+      <x:c r="T94" s="36"/>
+      <x:c r="U94" s="36"/>
+      <x:c r="V94" s="38" t="str">
         <x:f>IF(B94="","","https://hlctex.com/textile/products/"&amp;B94&amp;"/")</x:f>
       </x:c>
-      <x:c r="U94" s="38" t="str">
+      <x:c r="W94" s="38" t="str">
         <x:f>IF(B94="","",IF(A94&lt;&gt;"YES","未发布",IF(OR(C94="",D94="",J94=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V94" s="36"/>
+      <x:c r="X94" s="36"/>
     </x:row>
     <x:row r="95" ht="42" customHeight="1">
       <x:c r="A95" s="36"/>
@@ -3539,13 +3737,15 @@
       <x:c r="Q95" s="36"/>
       <x:c r="R95" s="36"/>
       <x:c r="S95" s="36"/>
-      <x:c r="T95" s="38" t="str">
+      <x:c r="T95" s="36"/>
+      <x:c r="U95" s="36"/>
+      <x:c r="V95" s="38" t="str">
         <x:f>IF(B95="","","https://hlctex.com/textile/products/"&amp;B95&amp;"/")</x:f>
       </x:c>
-      <x:c r="U95" s="38" t="str">
+      <x:c r="W95" s="38" t="str">
         <x:f>IF(B95="","",IF(A95&lt;&gt;"YES","未发布",IF(OR(C95="",D95="",J95=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V95" s="36"/>
+      <x:c r="X95" s="36"/>
     </x:row>
     <x:row r="96" ht="42" customHeight="1">
       <x:c r="A96" s="36"/>
@@ -3567,13 +3767,15 @@
       <x:c r="Q96" s="36"/>
       <x:c r="R96" s="36"/>
       <x:c r="S96" s="36"/>
-      <x:c r="T96" s="38" t="str">
+      <x:c r="T96" s="36"/>
+      <x:c r="U96" s="36"/>
+      <x:c r="V96" s="38" t="str">
         <x:f>IF(B96="","","https://hlctex.com/textile/products/"&amp;B96&amp;"/")</x:f>
       </x:c>
-      <x:c r="U96" s="38" t="str">
+      <x:c r="W96" s="38" t="str">
         <x:f>IF(B96="","",IF(A96&lt;&gt;"YES","未发布",IF(OR(C96="",D96="",J96=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V96" s="36"/>
+      <x:c r="X96" s="36"/>
     </x:row>
     <x:row r="97" ht="42" customHeight="1">
       <x:c r="A97" s="36"/>
@@ -3595,13 +3797,15 @@
       <x:c r="Q97" s="36"/>
       <x:c r="R97" s="36"/>
       <x:c r="S97" s="36"/>
-      <x:c r="T97" s="38" t="str">
+      <x:c r="T97" s="36"/>
+      <x:c r="U97" s="36"/>
+      <x:c r="V97" s="38" t="str">
         <x:f>IF(B97="","","https://hlctex.com/textile/products/"&amp;B97&amp;"/")</x:f>
       </x:c>
-      <x:c r="U97" s="38" t="str">
+      <x:c r="W97" s="38" t="str">
         <x:f>IF(B97="","",IF(A97&lt;&gt;"YES","未发布",IF(OR(C97="",D97="",J97=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V97" s="36"/>
+      <x:c r="X97" s="36"/>
     </x:row>
     <x:row r="98" ht="42" customHeight="1">
       <x:c r="A98" s="36"/>
@@ -3623,13 +3827,15 @@
       <x:c r="Q98" s="36"/>
       <x:c r="R98" s="36"/>
       <x:c r="S98" s="36"/>
-      <x:c r="T98" s="38" t="str">
+      <x:c r="T98" s="36"/>
+      <x:c r="U98" s="36"/>
+      <x:c r="V98" s="38" t="str">
         <x:f>IF(B98="","","https://hlctex.com/textile/products/"&amp;B98&amp;"/")</x:f>
       </x:c>
-      <x:c r="U98" s="38" t="str">
+      <x:c r="W98" s="38" t="str">
         <x:f>IF(B98="","",IF(A98&lt;&gt;"YES","未发布",IF(OR(C98="",D98="",J98=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V98" s="36"/>
+      <x:c r="X98" s="36"/>
     </x:row>
     <x:row r="99" ht="42" customHeight="1">
       <x:c r="A99" s="36"/>
@@ -3651,13 +3857,15 @@
       <x:c r="Q99" s="36"/>
       <x:c r="R99" s="36"/>
       <x:c r="S99" s="36"/>
-      <x:c r="T99" s="38" t="str">
+      <x:c r="T99" s="36"/>
+      <x:c r="U99" s="36"/>
+      <x:c r="V99" s="38" t="str">
         <x:f>IF(B99="","","https://hlctex.com/textile/products/"&amp;B99&amp;"/")</x:f>
       </x:c>
-      <x:c r="U99" s="38" t="str">
+      <x:c r="W99" s="38" t="str">
         <x:f>IF(B99="","",IF(A99&lt;&gt;"YES","未发布",IF(OR(C99="",D99="",J99=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V99" s="36"/>
+      <x:c r="X99" s="36"/>
     </x:row>
     <x:row r="100" ht="42" customHeight="1">
       <x:c r="A100" s="36"/>
@@ -3679,13 +3887,15 @@
       <x:c r="Q100" s="36"/>
       <x:c r="R100" s="36"/>
       <x:c r="S100" s="36"/>
-      <x:c r="T100" s="38" t="str">
+      <x:c r="T100" s="36"/>
+      <x:c r="U100" s="36"/>
+      <x:c r="V100" s="38" t="str">
         <x:f>IF(B100="","","https://hlctex.com/textile/products/"&amp;B100&amp;"/")</x:f>
       </x:c>
-      <x:c r="U100" s="38" t="str">
+      <x:c r="W100" s="38" t="str">
         <x:f>IF(B100="","",IF(A100&lt;&gt;"YES","未发布",IF(OR(C100="",D100="",J100=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V100" s="36"/>
+      <x:c r="X100" s="36"/>
     </x:row>
     <x:row r="101" ht="42" customHeight="1">
       <x:c r="A101" s="36"/>
@@ -3707,13 +3917,15 @@
       <x:c r="Q101" s="36"/>
       <x:c r="R101" s="36"/>
       <x:c r="S101" s="36"/>
-      <x:c r="T101" s="38" t="str">
+      <x:c r="T101" s="36"/>
+      <x:c r="U101" s="36"/>
+      <x:c r="V101" s="38" t="str">
         <x:f>IF(B101="","","https://hlctex.com/textile/products/"&amp;B101&amp;"/")</x:f>
       </x:c>
-      <x:c r="U101" s="38" t="str">
+      <x:c r="W101" s="38" t="str">
         <x:f>IF(B101="","",IF(A101&lt;&gt;"YES","未发布",IF(OR(C101="",D101="",J101=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V101" s="36"/>
+      <x:c r="X101" s="36"/>
     </x:row>
     <x:row r="102" ht="42" customHeight="1">
       <x:c r="A102" s="36"/>
@@ -3735,13 +3947,15 @@
       <x:c r="Q102" s="36"/>
       <x:c r="R102" s="36"/>
       <x:c r="S102" s="36"/>
-      <x:c r="T102" s="38" t="str">
+      <x:c r="T102" s="36"/>
+      <x:c r="U102" s="36"/>
+      <x:c r="V102" s="38" t="str">
         <x:f>IF(B102="","","https://hlctex.com/textile/products/"&amp;B102&amp;"/")</x:f>
       </x:c>
-      <x:c r="U102" s="38" t="str">
+      <x:c r="W102" s="38" t="str">
         <x:f>IF(B102="","",IF(A102&lt;&gt;"YES","未发布",IF(OR(C102="",D102="",J102=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V102" s="36"/>
+      <x:c r="X102" s="36"/>
     </x:row>
     <x:row r="103" ht="42" customHeight="1">
       <x:c r="A103" s="36"/>
@@ -3763,13 +3977,15 @@
       <x:c r="Q103" s="36"/>
       <x:c r="R103" s="36"/>
       <x:c r="S103" s="36"/>
-      <x:c r="T103" s="38" t="str">
+      <x:c r="T103" s="36"/>
+      <x:c r="U103" s="36"/>
+      <x:c r="V103" s="38" t="str">
         <x:f>IF(B103="","","https://hlctex.com/textile/products/"&amp;B103&amp;"/")</x:f>
       </x:c>
-      <x:c r="U103" s="38" t="str">
+      <x:c r="W103" s="38" t="str">
         <x:f>IF(B103="","",IF(A103&lt;&gt;"YES","未发布",IF(OR(C103="",D103="",J103=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V103" s="36"/>
+      <x:c r="X103" s="36"/>
     </x:row>
     <x:row r="104" ht="42" customHeight="1">
       <x:c r="A104" s="37"/>
@@ -3791,25 +4007,27 @@
       <x:c r="Q104" s="37"/>
       <x:c r="R104" s="37"/>
       <x:c r="S104" s="37"/>
-      <x:c r="T104" s="39" t="str">
+      <x:c r="T104" s="37"/>
+      <x:c r="U104" s="37"/>
+      <x:c r="V104" s="39" t="str">
         <x:f>IF(B104="","","https://hlctex.com/textile/products/"&amp;B104&amp;"/")</x:f>
       </x:c>
-      <x:c r="U104" s="39" t="str">
+      <x:c r="W104" s="39" t="str">
         <x:f>IF(B104="","",IF(A104&lt;&gt;"YES","未发布",IF(OR(C104="",D104="",J104=""),"缺少必填项","可生成")))</x:f>
       </x:c>
-      <x:c r="V104" s="37"/>
+      <x:c r="X104" s="37"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:V1"/>
-    <x:mergeCell ref="A2:V2"/>
+    <x:mergeCell ref="A1:X1"/>
+    <x:mergeCell ref="A2:X2"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="A5:A104">
     <x:cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <x:formula>"YES"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="U5:U104">
+  <x:conditionalFormatting sqref="W5:W104">
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="缺少"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
@@ -3819,7 +4037,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7ddb837096f4004"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6eed3f5a5e734d49"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5775,7 +5993,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ef881c272164fd0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd99905ebee5b4cd7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6007,7 +6225,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86339c6b855340ed"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8aeab3ccca754278"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6665,7 +6883,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R121085129ff94479"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54a3843f9b244614"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>